<commit_message>
Lead extraction 2026-08-26 (weekly, uta)
</commit_message>
<xml_diff>
--- a/UT/uta/2026-08-26.xlsx
+++ b/UT/uta/2026-08-26.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,11 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Posted Date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Property Value</t>
         </is>
       </c>
@@ -508,6 +513,11 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>$410,900</t>
         </is>
       </c>
@@ -549,10 +559,268 @@
           <t>initial L matches deceased's own name 'Lynn'</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/person/carol-lynn-pearson-(perry)-11637372</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>$708,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Gwen Rodeback Smith</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SMITH, GWEN R</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>51:310:0002</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>218 N 1140 EAST</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PAYSON</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>initial R matches deceased's own name 'Rodeback'</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>$279,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Michael James Frost</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FROST, MICHAEL J</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>08:112:0013</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>775 S 500 EAST</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PAYSON</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'James'</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/person/michael-james-frost-62162943</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>$468,200</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>George Joseph Woffinden</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WOFFINDEN, GEORGE J</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>19:027:0043</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1435 S 300 WEST</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OREM</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'Joseph'</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>$251,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>George Joseph Woffinden</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>WOFFINDEN, GEORGE J</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>19:027:0044</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>OREM</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Utah County</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'Joseph'</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>$258,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>George Joseph Woffinden</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>WOFFINDEN, GEORGE J</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>19:027:0106</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1435 S 300 WEST</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OREM</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'Joseph'</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>$564,300</t>
         </is>
       </c>
     </row>

</xml_diff>